<commit_message>
UP cross-check: SOC 2 out of scope, AppSource per PZ1, group 60131, risk crosswalk, appendix B as accepted decisions, Excel notes, rebuild
</commit_message>
<xml_diff>
--- a/ЛР2-3_Объем_рынка/Excel/ЛР2-3_2_сверху_вниз_снизу_вверх_TableMind.xlsx
+++ b/ЛР2-3_Объем_рынка/Excel/ЛР2-3_2_сверху_вниз_снизу_вверх_TableMind.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-3ab569\ЛР2-3_Объем_рынка\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-57ce20\ЛР2-3_Объем_рынка\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02EC20DF-776C-4609-9D4A-EDBDFD129358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D98DE4-FC8B-44C2-8455-98D03C830B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Методика" sheetId="1" r:id="rId1"/>
@@ -887,7 +887,7 @@
     <t>PerfectXL от 69 EUR, Numerous 10 USD, Rows 8 USD, Shortcut 100 USD, Copilot 18 USD (03.10.2026)</t>
   </si>
   <si>
-    <t>Нет доступа к рекламным кабинетам: ДОСНЯТЬ тестовые кампании</t>
+    <t>Нет доступа к рекламным кабинетам: использованы модельные показатели (допущение Д-33)</t>
   </si>
 </sst>
 </file>
@@ -1144,13 +1144,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="6" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1159,6 +1152,13 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1336,28 +1336,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="4" spans="1:8" ht="40.9">
       <c r="A4" s="1" t="s">
@@ -1521,24 +1521,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="2" spans="1:6" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
     </row>
     <row r="4" spans="1:6" ht="13.05" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -1816,26 +1816,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
     </row>
     <row r="2" spans="1:7" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
     </row>
     <row r="4" spans="1:7" ht="13.05" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -2079,32 +2079,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
     </row>
     <row r="2" spans="1:10" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
     </row>
     <row r="4" spans="1:10" ht="13.05" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -2391,38 +2391,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
     </row>
     <row r="2" spans="1:13" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="37"/>
-      <c r="M2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
+      <c r="M2" s="40"/>
     </row>
     <row r="4" spans="1:13" ht="13.05" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -2496,13 +2496,13 @@
         <v>137211.97009990257</v>
       </c>
       <c r="J5" s="24">
-        <f>I5/SUM($I$5:$I$16)</f>
+        <f t="shared" ref="J5:J11" si="2">I5/SUM($I$5:$I$16)</f>
         <v>0.14949327113336192</v>
       </c>
       <c r="K5" s="16" t="s">
         <v>252</v>
       </c>
-      <c r="L5" s="39">
+      <c r="L5" s="36">
         <v>46298</v>
       </c>
       <c r="M5" s="28" t="s">
@@ -2540,13 +2540,13 @@
         <v>107759.75295240001</v>
       </c>
       <c r="J6" s="24">
-        <f>I6/SUM($I$5:$I$16)</f>
+        <f t="shared" si="2"/>
         <v>0.11740490245601883</v>
       </c>
       <c r="K6" s="16" t="s">
         <v>256</v>
       </c>
-      <c r="L6" s="39">
+      <c r="L6" s="36">
         <v>46298</v>
       </c>
       <c r="M6" s="28" t="s">
@@ -2584,13 +2584,13 @@
         <v>36421.232535552597</v>
       </c>
       <c r="J7" s="24">
-        <f>I7/SUM($I$5:$I$16)</f>
+        <f t="shared" si="2"/>
         <v>3.9681153083687512E-2</v>
       </c>
       <c r="K7" s="16" t="s">
         <v>259</v>
       </c>
-      <c r="L7" s="39">
+      <c r="L7" s="36">
         <v>46298</v>
       </c>
       <c r="M7" s="28" t="s">
@@ -2628,13 +2628,13 @@
         <v>94737.990815733603</v>
       </c>
       <c r="J8" s="24">
-        <f>I8/SUM($I$5:$I$16)</f>
+        <f t="shared" si="2"/>
         <v>0.10321761386659423</v>
       </c>
       <c r="K8" s="16" t="s">
         <v>261</v>
       </c>
-      <c r="L8" s="39">
+      <c r="L8" s="36">
         <v>46298</v>
       </c>
       <c r="M8" s="28" t="s">
@@ -2672,13 +2672,13 @@
         <v>46467.755357184004</v>
       </c>
       <c r="J9" s="24">
-        <f>I9/SUM($I$5:$I$16)</f>
+        <f t="shared" si="2"/>
         <v>5.0626900448353607E-2</v>
       </c>
       <c r="K9" s="16" t="s">
         <v>263</v>
       </c>
-      <c r="L9" s="39">
+      <c r="L9" s="36">
         <v>46298</v>
       </c>
       <c r="M9" s="28" t="s">
@@ -2708,7 +2708,7 @@
         <v>0.8</v>
       </c>
       <c r="H10" s="22">
-        <f t="shared" ref="H10:H11" si="2">C10*D10*E10*F10*G10</f>
+        <f t="shared" ref="H10:H11" si="3">C10*D10*E10*F10*G10</f>
         <v>5631.726821990399</v>
       </c>
       <c r="I10" s="22">
@@ -2716,13 +2716,13 @@
         <v>67580.721863884784</v>
       </c>
       <c r="J10" s="24">
-        <f>I10/SUM($I$5:$I$16)</f>
+        <f t="shared" si="2"/>
         <v>7.3629605125779193E-2</v>
       </c>
       <c r="K10" s="16" t="s">
         <v>265</v>
       </c>
-      <c r="L10" s="39">
+      <c r="L10" s="36">
         <v>46298</v>
       </c>
       <c r="M10" s="28" t="s">
@@ -2752,7 +2752,7 @@
         <v>0.8</v>
       </c>
       <c r="H11" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6331.1611225199995</v>
       </c>
       <c r="I11" s="22">
@@ -2760,13 +2760,13 @@
         <v>75973.933470239994</v>
       </c>
       <c r="J11" s="24">
-        <f>I11/SUM($I$5:$I$16)</f>
+        <f t="shared" si="2"/>
         <v>8.2774059923964693E-2</v>
       </c>
       <c r="K11" s="16" t="s">
         <v>267</v>
       </c>
-      <c r="L11" s="39">
+      <c r="L11" s="36">
         <v>46298</v>
       </c>
       <c r="M11" s="28" t="s">
@@ -2810,7 +2810,7 @@
       <c r="K12" s="16" t="s">
         <v>269</v>
       </c>
-      <c r="L12" s="39">
+      <c r="L12" s="36">
         <v>46298</v>
       </c>
       <c r="M12" s="28" t="s">
@@ -2854,7 +2854,7 @@
       <c r="K13" s="16" t="s">
         <v>271</v>
       </c>
-      <c r="L13" s="39">
+      <c r="L13" s="36">
         <v>46298</v>
       </c>
       <c r="M13" s="28" t="s">
@@ -2898,7 +2898,7 @@
       <c r="K14" s="16" t="s">
         <v>273</v>
       </c>
-      <c r="L14" s="39">
+      <c r="L14" s="36">
         <v>46298</v>
       </c>
       <c r="M14" s="28" t="s">
@@ -2942,7 +2942,7 @@
       <c r="K15" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="L15" s="39">
+      <c r="L15" s="36">
         <v>46298</v>
       </c>
       <c r="M15" s="28" t="s">
@@ -2986,7 +2986,7 @@
       <c r="K16" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="L16" s="39">
+      <c r="L16" s="36">
         <v>46298</v>
       </c>
       <c r="M16" s="28" t="s">
@@ -3044,26 +3044,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
     </row>
     <row r="2" spans="1:7" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
     </row>
     <row r="4" spans="1:7" ht="13.05" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -3361,28 +3361,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>146</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="4" spans="1:8" ht="13.05" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -3589,28 +3589,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="4" spans="1:8" ht="13.05" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -3833,28 +3833,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="39" t="s">
         <v>188</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="12" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="4" spans="1:8" ht="13.05" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -3895,7 +3895,7 @@
       <c r="D5" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="E5" s="40">
+      <c r="E5" s="37">
         <v>46298</v>
       </c>
       <c r="F5" s="13" t="s">
@@ -3921,7 +3921,7 @@
       <c r="D6" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="E6" s="40">
+      <c r="E6" s="37">
         <v>46298</v>
       </c>
       <c r="F6" s="13" t="s">
@@ -3947,7 +3947,7 @@
       <c r="D7" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="E7" s="40">
+      <c r="E7" s="37">
         <v>46298</v>
       </c>
       <c r="F7" s="13" t="s">
@@ -3971,7 +3971,7 @@
         <v>213</v>
       </c>
       <c r="D8" s="16"/>
-      <c r="E8" s="40">
+      <c r="E8" s="37">
         <v>46298</v>
       </c>
       <c r="F8" s="13" t="s">
@@ -3995,7 +3995,7 @@
         <v>218</v>
       </c>
       <c r="D9" s="16"/>
-      <c r="E9" s="40">
+      <c r="E9" s="37">
         <v>46298</v>
       </c>
       <c r="F9" s="13" t="s">
@@ -4008,7 +4008,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="54">
+    <row r="10" spans="1:8" ht="67.5">
       <c r="A10" s="14" t="s">
         <v>221</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>223</v>
       </c>
       <c r="D10" s="17"/>
-      <c r="E10" s="41">
+      <c r="E10" s="38">
         <v>46298</v>
       </c>
       <c r="F10" s="15" t="s">

</xml_diff>

<commit_message>
reports: model-based data described as calculation models, no process notes; rebuild
</commit_message>
<xml_diff>
--- a/ЛР2-3_Объем_рынка/Excel/ЛР2-3_2_сверху_вниз_снизу_вверх_TableMind.xlsx
+++ b/ЛР2-3_Объем_рынка/Excel/ЛР2-3_2_сверху_вниз_снизу_вверх_TableMind.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-57ce20\ЛР2-3_Объем_рынка\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-89518d\ЛР2-3_Объем_рынка\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D98DE4-FC8B-44C2-8455-98D03C830B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45376034-93EC-4A5F-8A12-9B2BDF6AFD59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -887,7 +887,7 @@
     <t>PerfectXL от 69 EUR, Numerous 10 USD, Rows 8 USD, Shortcut 100 USD, Copilot 18 USD (03.10.2026)</t>
   </si>
   <si>
-    <t>Нет доступа к рекламным кабинетам: использованы модельные показатели (допущение Д-33)</t>
+    <t>Нет доступа к рекламным кабинетам: использованы расчетные показатели (допущение Д-33)</t>
   </si>
 </sst>
 </file>

</xml_diff>